<commit_message>
run-006 delivery + run-007 Reissue flow (Stage 1 approved, Stage 2 in progress)
run-006 (Auto Reissue checkbox, Agency + Branch):
- Stage 2 discovery findings FINDING-013..017, investigation of supplier/credential dependency
- Stage 3 test cases TC-AGENCY-061..094, TC-BR-083..112 with traceability and coverage
- Stage 4M manual execution results, report and evidence

run-007 (Supplier Feature reissue, shared scope reissue-flow, Sabre Staging):
- Stage 1 Project Context approved (Rev 2, decisions D-1..D-13)
- Stage 2 discovery evidence: Admin/Portal flow up to Review & Pay,
  Sabre -> core service -> Admin API -> screen mapping comparison,
  CL-1 check (DS-2 pending), FINDING-R01 Itinerary time-zone shift
- Handoff note for resuming on another device

Credentials stay in the git-ignored credentials.json; staged files scanned for secrets.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/platform_core_data/modules/agency/test_design/TestCases_Agency.xlsx
+++ b/platform_core_data/modules/agency/test_design/TestCases_Agency.xlsx
@@ -60,7 +60,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3787,6 +3787,1950 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Auto Reissue is unchecked by default on Add Agency</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a new Agency form shows the Auto Reissue checkbox unchecked.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Logged in to Admin (`http://192.168.1.60`). Nothing is saved by this case.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Admin → Agency**. | 2. Click **Add**. | 3. Scroll to **Agency Features**. | 4. Leave the page without saving.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Auto Reissue** is shown under Agency Features and is unchecked. **Auto Reissue Credentials** is not shown.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ticking Auto Reissue shows the credentials picker</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that Auto Reissue Credentials appears only while Auto Reissue is ticked.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">On the Add Agency form. Nothing is saved by this case.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Tick **Auto Reissue**. | 2. Untick **Auto Reissue**. | 3. Leave the page without saving.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">After step 1, **Auto Reissue Credentials** appears. After step 2, it is hidden.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Turn Auto Reissue on for an Agency and save</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that Auto Reissue and one credential are saved and shown again when the Agency is reopened.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Agency | AGN9780 |
+| Auto Reissue Credentials | the first option offered |</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Admin → Agency**, search `AGN9780` with Status **Both**. | 2. Click the edit pen. | 3. Tick **Auto Reissue**. | 4. In **Auto Reissue Credentials**, select the first option. | 5. Enter a remark. | 6. Click **Approve**. | 7. Reopen AGN9780.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Auto Reissue** is ticked and the credential chosen in step 4 is shown in **Auto Reissue Credentials**.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The edit form's **Approve** saves and approves in one step, so the Agency never goes Inactive (`PO-24`). Restore afterwards: untick Auto Reissue and Approve (or run TC-AGENCY-073 next).</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Auto Reissue change waits for approval after Send For Approval</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an Auto Reissue change sent for approval takes effect only after it is approved.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Tick **Auto Reissue** and select one credential. | 3. Enter a remark. | 4. Click **Send For Approval**. | 5. Search AGN9780 with Status **Both** and read its row. | 6. Approve the row, entering a remark. | 7. Reopen AGN9780.</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">After step 5, the row shows **Inactive** and **Pending for approval**. After step 6, it shows **Active** and **Approved**. After step 7, Auto Reissue is ticked with the chosen credential.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Regression</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Inactive while pending is normal (`PO-24`). Don't run booking checks while AGN9780 is pending. Restore: untick and Approve.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Auto Reissue on with no credential shows "Required"</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the form will not save Auto Reissue on without a credential.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Tick **Auto Reissue**. | 3. Leave **Auto Reissue Credentials** empty. | 4. Enter a remark. | 5. Click **Send For Approval**.</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">"Required" appears under **Auto Reissue Credentials**. The Agency is not saved: its row stays Approved and Auto Reissue stays off.</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-EmptyValues</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API rejects Auto Reissue on with an empty credential list</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the API rejects Auto Reissue on with no credentials.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `true` · `reissueCredentials`: `[]`</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set `autoReissueEnabled` and `reissueCredentials` to the Test Data values. Leave every other field as captured. | 2. Send the request. | 3. Search AGN9780 in Admin → Agency (Status: Both) and read its row.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The response is **400** with message "Select at least one eligible credential". AGN9780 is unchanged.</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-EmptyValues</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API keeps the saved credentials when Auto Reissue is sent off with others</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that credentials sent with Auto Reissue off are replaced by the Agency's saved valid selection.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved, Auto Reissue off, with a saved credential `{STORED}` (read it with the GET in §0.3).</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `false` · `reissueCredentials`: `[{"credentialId": &lt;any ID other than {STORED}&gt;}]`</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set the two fields to the Test Data values. | 2. Send the request. | 3. Approve AGN9780 from the Agency grid, entering a remark. | 4. Read AGN9780 with the GET in §0.3.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The request succeeds. The GET returns `autoReissueEnabled: false` and `reissueCredentials` equal to `{STORED}`, not the ID that was sent.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">This request is a real save, so AGN9780 goes to Pending until step 3.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API rejects a credential without an ID</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the API rejects a reissue credential that has no ID.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `true` · `reissueCredentials`: `[{}]`</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set `autoReissueEnabled` and `reissueCredentials` to the Test Data values. Leave every other field as captured. | 2. Send the request. | 3. Search AGN9780 in Admin → Agency (Status: Both) and read its row.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The response is **400** with message "Every auto-reissue credential must have an ID". AGN9780 is unchanged.</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API rejects an unknown credential ID</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the API rejects a credential ID that does not exist.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `true` · `reissueCredentials`: `[{"credentialId": 999999}]`</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set `autoReissueEnabled` and `reissueCredentials` to the Test Data values. Leave every other field as captured. | 2. Send the request. | 3. Search AGN9780 in Admin → Agency (Status: Both) and read its row.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The response is **400** with message "Every auto-reissue credential must exist and be active". AGN9780 is unchanged.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API rejects an inactive credential</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the API rejects a credential that exists but is inactive.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `true` · `reissueCredentials`: `[{"credentialId": {INACTIVE_ID}}]`</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set `autoReissueEnabled` and `reissueCredentials` to the Test Data values. Leave every other field as captured. | 2. Send the request. | 3. Search AGN9780 in Admin → Agency (Status: Both) and read its row.</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The response is **400** with message "Every auto-reissue credential must exist and be active". AGN9780 is unchanged.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs, Assumption-based</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Needs `{INACTIVE_ID}`: an inactive supplier credential mapped to AGN9780.** Discovery found none on `.60`. **Set it up with TC-AGENCY-092** (the user's go-ahead to make a credential inactive) and run this case inside that inactive window. Without it, record **Blocked**, not Failed.</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API rejects duplicate credential IDs</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the API rejects the same credential sent twice.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `true` · `reissueCredentials`: `[{"credentialId": X}, {"credentialId": X}]`, where X is a credential offered in AGN9780's picker</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set `autoReissueEnabled` and `reissueCredentials` to the Test Data values. Leave every other field as captured. | 2. Send the request. | 3. Search AGN9780 in Admin → Agency (Status: Both) and read its row.</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The response is **400** with message "Auto-reissue credentials must not contain duplicates". AGN9780 is unchanged.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">API rejects a credential not assigned to the Agency</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an Agency cannot be given a reissue credential it is not assigned.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The `{AGENCY_SAVE_REQUEST}` fixture is loaded in Postman (§0.3). AGN9780 is Approved.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">`autoReissueEnabled`: `true` · `reissueCredentials`: `[{"credentialId": Y}]`, where Y is a supported credential **not** offered in AGN9780's picker (e.g. 287 or 289 — check first)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. In `{AGENCY_SAVE_REQUEST}`, set `autoReissueEnabled` and `reissueCredentials` to the Test Data values. Leave every other field as captured. | 2. Send the request. | 3. Search AGN9780 in Admin → Agency (Status: Both) and read its row.</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The response is **400** with message "Each auto-reissue credential must be mapped to this organization". AGN9780 is unchanged.</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs, Permissions</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Turning Auto Reissue off keeps the saved credentials</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that credentials saved with Auto Reissue on return when it is turned on again.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved, Auto Reissue on, with credential `{C}` (e.g. after TC-AGENCY-063).</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Untick **Auto Reissue**. | 3. Enter a remark and click **Approve**. | 4. Reopen AGN9780. | 5. Tick **Auto Reissue**. | 6. Read **Auto Reissue Credentials**. | 7. Leave the page without saving.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">After step 4, Auto Reissue is unticked. After step 6, the picker already shows `{C}`.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, Regression</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Leaves AGN9780 off, which is its restore state.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Agency picker offers only credentials the Agency itself holds</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Agency's Auto Reissue picker lists only credentials chosen on that Agency, not other credentials its Branch has.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">BRN265 has at least one supported GDS credential that is **not** chosen in AGN9780's PCC tabs (record it as `{BRANCH_ONLY}`). The credentials chosen in AGN9780's PCC tabs are recorded. Nothing is saved by this case.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Tick **Auto Reissue**. | 3. Open **Auto Reissue Credentials** and record every option. | 4. Leave the page without saving.</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Every option is a credential chosen in AGN9780's own PCC tabs. `{BRANCH_ONLY}` is not offered.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Integration, Business-Rule</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Corrected by the user on 2026-09-25: the picker offers the credentials the **Agency** holds, not everything its Branch holds. The Agency's credentials are a subset of the Branch's (`PO-16`, `PO-27`). Rewritten on 2026-09-25 (was *"…credentials its Branch holds"*); Review was already Pending. Discovery hasn't settled this: on 2026-09-23 the picker also offered 313 (NDCsbr) while NDCsbr looked unticked on AGN9780 (agency Timeline run-006 21:38). This case checks it directly.</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reading the Agency drops a credential that became invalid</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a saved credential that became invalid is removed when the Agency is read, while Auto Reissue stays on.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on and a saved credential that has since become inactive, unassigned or unsupported.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Reopen AGN9780. | 2. Read **Auto Reissue** and **Auto Reissue Credentials**.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The invalid credential is no longer listed. **Auto Reissue** stays ticked, even if no credential is left.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Assumption-based</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Reaching the precondition needs a supplier or credential change that this run is not granted (RSK-012).** **TC-AGENCY-092 sets up this state** (with the user's go-ahead); run this case inside its inactive window. Otherwise record **Blocked**.</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admin shows Reissue for an Agency booking when Auto Reissue is on</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Admin Itinerary shows Reissue when the booking's Agency has Auto Reissue on.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved). Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre, Status Booked) is not locked by another user.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `NDCEG-BR-F260924EAzzYT` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is shown.</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admin hides Reissue for an Agency booking when Auto Reissue is off</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Admin Itinerary hides Reissue when the booking's Agency has Auto Reissue off.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue off (Approved). Booking `NDCEG-BR-F260924EAzzYT` is not locked by another user.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `NDCEG-BR-F260924EAzzYT` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown. **Manual Reissue** is still shown.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative, Smoke</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`). Manual Reissue does not depend on this checkbox.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Branch Auto Reissue on does not enable an Agency booking</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a Branch with Auto Reissue on does not show Reissue on its Agency's booking when the Agency is off.</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">BRN265 has Auto Reissue on. AGN9780 has Auto Reissue off. Both Approved.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `NDCEG-BR-F260924EAzzYT` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Integration</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Portal shows Reissue when the Agency has Auto Reissue on</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Portal shows Reissue on the Agency's booking when Auto Reissue is on.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved). The AGN9780 Portal login is available.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Log in to the Portal (`http://192.168.1.60:9500`) with agency code `AGN9780`. | 2. Open **My Booking** and click **Search**. | 3. Click the **Order Id** of booking `NDCEG-BR-F260924EAzzYT`. | 4. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is shown.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No lock is needed on the Portal (`PO-25`). Never click Reissue.</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Portal hides Reissue when the Agency has Auto Reissue off</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Portal hides Reissue on the Agency's booking when Auto Reissue is off.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue off (Approved). The AGN9780 Portal login is available.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Log in to the Portal (`http://192.168.1.60:9500`) with agency code `AGN9780`. | 2. Open **My Booking** and click **Search**. | 3. Click the **Order Id** of booking `NDCEG-BR-F260924EAzzYT`. | 4. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative, Smoke</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-081</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Portal shows Reissue without a lock and offers no Manual Reissue</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Portal booking has no lock control and no Manual Reissue.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved).</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Log in to the Portal (`http://192.168.1.60:9500`) with agency code `AGN9780`. | 2. Open **My Booking** and click **Search**. | 3. Click the **Order Id** of booking `NDCEG-BR-F260924EAzzYT`. | 4. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Created By** card has no lock control. **Reissue** is shown. **Manual Reissue** is not shown.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Regression</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Confirmed intended by the user on 2026-09-24 (FINDING-016, `PO-25`).</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-082</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reissue shows even if the booking's credential is not selected</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Reissue button depends on the checkbox only, not on which credentials are selected.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved), with a selected credential that is **not** the booking's credential (the booking is on "Sabre Staging").</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `NDCEG-BR-F260924EAzzYT` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is shown.</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Business-Rule</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The credential check happens only when Reissue is clicked, and belongs to the `reissue-flow` scope (`PO-22`). Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-083</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A booking made on behalf of the Agency follows the Agency's checkbox</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a booking made on behalf of an Agency hides Reissue when that Agency is off, even if the Branch is on.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A Booked booking made by Admin or the Branch **on behalf of AGN9780**, supplied by the user (`{ONBEHALF_REF}`). BRN265 on, AGN9780 off, both Approved.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `{ONBEHALF_REF}` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Integration, Assumption-based</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The platform never books; the user supplies `{ONBEHALF_REF}`. Without it, record **Blocked — Awaiting User Booking**. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-084</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A booking not in Booked status does not show Reissue</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that Reissue is hidden for an Agency booking whose status is not Booked.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A booking under AGN9780 in a status other than Booked (e.g. Cancelled), supplied by the user (`{NOTBOOKED_REF}`). AGN9780 on (Approved).</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `{NOTBOOKED_REF}` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative, Assumption-based</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Without `{NOTBOOKED_REF}`, record **Blocked — Awaiting User Booking**. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-085</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Which value the Itinerary uses while an Auto Reissue change is pending</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Find out whether the Itinerary follows the approved or the pending Auto Reissue value.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780, tick **Auto Reissue**, select one credential, enter a remark. | 2. Click **Send For Approval**. Do not approve yet. | 3. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 4. Click the **Flight** tab. | 5. Enter Booking Reference `NDCEG-BR-F260924EAzzYT` and click **Search**. | 6. Open the booking from the result row. | 7. Click the lock icon on the **Created By** card. | 8. Click **View Passenger Details**. | 9. Record whether **Reissue** is shown. | 10. Reject or approve the pending change, then restore AGN9780 to off.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The tester records whether **Reissue** is shown while the change is pending, and the reviewer confirms whether that is intended.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Exploratory, Assumption-based</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Exploratory: no fixed pass/fail. Opens RSK-013. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-086</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Updating an Agency without touching Auto Reissue still works</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an ordinary Agency update still saves and leaves Auto Reissue unchanged.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved. Its Auto Reissue value and credentials are recorded.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Change only the **Remarks** text. | 3. Click **Approve**. | 4. Reopen AGN9780.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The update is saved and approved. **Auto Reissue** and **Auto Reissue Credentials** are the same as recorded.</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Regression, Smoke</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-087</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Create an Agency with Auto Reissue on</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a new Agency can be created with Auto Reissue on and a credential.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The user has been asked and agrees to create one new Agency under BRN265 (`AUTH-AGENCY-CREATE-SelfCreated`). The Agency's other mandatory fields are ready.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Agency name | `RUN006_AR_Agency` |
+| Branch | BRN265 |
+| Auto Reissue Credentials | the first option offered |</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Admin → Agency → Add**. | 2. Fill the mandatory fields with Test Data, Branch BRN265. | 3. Tick **Auto Reissue** and select the first credential. | 4. Enter a remark and click **Send For Approval**. | 5. Approve the new Agency from the grid. | 6. Reopen the new Agency.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The new Agency shows **Auto Reissue** ticked with the chosen credential.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Creates a lasting record on STG.** Capture its code right after step 5. It can't be deleted.</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-088</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Create an Agency with Auto Reissue off</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a new Agency can be created with Auto Reissue left off.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The user has been asked and agrees to create one new Agency under BRN265. Its other mandatory fields are ready.</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Agency name | `RUN006_AR_Off_Agency` |
+| Branch | BRN265 |
+| Auto Reissue | left unchecked |</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Admin → Agency → Add**. | 2. Fill the mandatory fields with Test Data. | 3. Leave **Auto Reissue** unchecked. | 4. Enter a remark and click **Send For Approval**. | 5. Approve the new Agency from the grid, entering a remark. | 6. Reopen the new Agency.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The Agency is created and approved. **Auto Reissue** is unticked and **Auto Reissue Credentials** is not shown.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Creates a lasting record on STG.** Capture its code right after step 5.</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Edit an Agency with Auto Reissue off</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an Agency with Auto Reissue off saves without asking for a credential.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Leave **Auto Reissue** unticked. | 3. Change only the remark text. | 4. Click **Approve**. | 5. Reopen AGN9780.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The save succeeds with no "Required" message. **Auto Reissue** is still unticked.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Edit an Agency with Auto Reissue on</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that editing an Agency that has Auto Reissue on keeps it on with the same credential.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue on and credential `{C}` (e.g. after TC-AGENCY-063).</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Change only the remark text. | 3. Click **Approve**. | 4. Reopen AGN9780.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Auto Reissue** is still ticked and **Auto Reissue Credentials** still shows `{C}`.</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Regression</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Restore afterwards: untick Auto Reissue and Approve.</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">An Agency can only have suppliers its Branch has</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Agency's Product Access offers no supplier that its parent Branch lacks.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The suppliers on BRN265 are recorded. Nothing is saved by this case.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Edit AGN9780. | 2. Open **Product Access Details**. | 3. Record every supplier listed. | 4. Leave the page without saving.</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Every supplier listed for AGN9780 is one that BRN265 has. No other supplier can be selected.</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Integration, Permissions</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The Branch is the supplier ceiling for its Agencies (`PO-27`). The reverse direction is TC-BR-109.</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">An inactive credential leaves the Agency's Auto Reissue picker</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a reissue credential made inactive is dropped from the Agency's saved selection and picker, while Auto Reissue stays on.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A supported GDS credential `{CRED}` (e.g. a Galileo credential) that no other organisation uses, chosen in the PCC tabs of both BRN265 and AGN9780. AGN9780 has Auto Reissue on with `{CRED}` selected, Approved.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Master → Supplier → Supplier Credentials** and search `{CRED}`. | 2. Edit `{CRED}`, set its status to **Inactive**, and save. | 3. Open AGN9780 for edit (Admin → Agency). | 4. Read **Auto Reissue** and **Auto Reissue Credentials**. | 5. Open **Auto Reissue Credentials** and read the options. | 6. Leave the form without saving. | 7. Set `{CRED}` back to **Active** and save.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">After step 4, `{CRED}` is no longer in the saved selection, and **Auto Reissue** is still ticked. After step 5, `{CRED}` is not offered.</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Negative, Integration</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ask the user before running this case. It changes **shared master data** (Master → Supplier) on staging, which affects every organisation that uses it. Use only a supplier/credential that no other organisation uses, record the grant in the run's `SafetyAuthorizations.json` first, and **set it back to Active at the end**. Spec §4: "a selected credential that has become inactive … is removed; the checkbox stays on". Run TC-AGENCY-070 (S-5 inactive) between steps 2 and 7, since `{CRED}` is its missing precondition. Record exactly what is seen.</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">What the Agency's Auto Reissue picker shows when the supplier is made inactive</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Find out what happens to the Agency's Auto Reissue selection and picker when the credential's supplier is made inactive.</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">As TC-AGENCY-092, using a GDS supplier `{SUP}` that no other organisation uses. AGN9780 has Auto Reissue on with a `{SUP}` credential selected, Approved.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Master → Supplier → Supplier** and search `{SUP}`. | 2. Edit `{SUP}`, set its status to **Inactive**, and save. | 3. Open AGN9780 for edit. | 4. Read **Auto Reissue**, **Auto Reissue Credentials** and **Product Access Details**. | 5. Open **Auto Reissue Credentials** and read the options. | 6. Leave the form without saving. | 7. Set `{SUP}` back to **Active** and save.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The tester records what is shown in steps 4–5, and the reviewer confirms whether it is intended. Spec §4 suggests the `{SUP}` credential is dropped and not offered, with Auto Reissue still ticked.</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Exploratory, Integration</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ask the user before running this case. It changes **shared master data** (Master → Supplier) on staging, which affects every organisation that uses it. Use only a supplier/credential that no other organisation uses, record the grant in the run's `SafetyAuthorizations.json` first, and **set it back to Active at the end**. Exploratory: the specification covers an inactive **credential**, not an inactive **supplier**.</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Portal hides Reissue for an Agency booking on hold</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Portal does not show Reissue for an Agency booking whose status is On Hold.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved). Booking `NDCEG-BR-F251014N1oohh` (AGN9780, On Hold). The AGN9780 Portal login is available.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Log in to the Portal (`http://192.168.1.60:9500`) with agency code `AGN9780`. | 2. Open **My Booking** and click **Search**. | 3. Click the **Order Id** of booking `NDCEG-BR-F251014N1oohh`. | 4. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Added 2026-09-25 at the user's request ("check the appearance of the button in Admin and Portal"). The Admin side is TC-AGENCY-084. Only Status **Booked** shows Reissue (spec §5, `PO-24`). Never click **Reissue**, **Release PNR** or **Void / Cancel**.</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reissue: D-14 Reissue button display rule; drop five Exchange edge cases
- D-14 (six-condition Reissue button rule) recorded across reissue-flow,
  reissue-mapping, agency and branch contexts, test design and coverage;
  settles DS-2. reissue-flow test suite Revision 2.
- User story: removed Exchange edge cases 5.10-5.14 (missing Booking
  Reference / Order ID, Reissue History creation failure, original offer
  status update failure, total-vs-difference price persistence);
  renumbered 5.15-5.18 to 5.10-5.13.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/platform_core_data/modules/agency/test_design/TestCases_Agency.xlsx
+++ b/platform_core_data/modules/agency/test_design/TestCases_Agency.xlsx
@@ -60,7 +60,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="D77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection (`PO-28`)**. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre, credential 315, Status Booked) is not locked by another user.</t>
+          <t xml:space="preserve">**All six `PO-30` conditions hold.** AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection**. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). It is not locked by another user; step 5 locks it to you.</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
@@ -4688,12 +4688,12 @@
       </c>
       <c r="J77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — preconditions restated against the six `PO-30` conditions (adds the "Ticketed Document" bar, online booking, reissue-capable GDS and the lock). Expected result unchanged. Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L77" t="inlineStr" s="2">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 has Auto Reissue off (Approved). Booking `NDCEG-BR-F260924EAzzYT` is not locked by another user.</t>
+          <t xml:space="preserve">AGN9780 has Auto Reissue off (Approved), with Sabre Staging (315) still in its saved selection. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). It is not locked by another user; step 5 locks it to you. **Only `PO-30` condition (1) — the checkbox — is unmet.**</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
@@ -4745,12 +4745,12 @@
       </c>
       <c r="J78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">**Rev 2, 2026-09-27** — the clause *"Manual Reissue is still shown"* was removed: Manual Reissue is out of scope for this story (`PO-29`). Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 3, 2026-10-01** — preconditions restated so the checkbox is the only `PO-30` condition left unmet; the status note now requires the "Ticketed Document" bar too. Expected result unchanged. **Rev 2, 2026-09-27** — the clause *"Manual Reissue is still shown"* was removed: Manual Reissue is out of scope for this story (`PO-29`). Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L78" t="inlineStr" s="2">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="D79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">BRN265 has Auto Reissue on. AGN9780 has Auto Reissue off. Both Approved.</t>
+          <t xml:space="preserve">BRN265 has Auto Reissue on. AGN9780 has Auto Reissue off. Both Approved. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). Step 5 locks it to you, so only AGN9780's checkbox (`PO-30` condition 1) is unmet.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
@@ -4802,12 +4802,12 @@
       </c>
       <c r="J79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — preconditions restated against `PO-30`; the status note now requires the "Ticketed Document" bar too. Expected result unchanged. Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L79" t="inlineStr" s="2">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="D80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection (`PO-28`)**. The AGN9780 Portal login is available.</t>
+          <t xml:space="preserve">**Every `PO-30` condition except the lock holds** — the Portal has no lock and needs none (`PO-25`). AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection**. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). The AGN9780 Portal login is available.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -4859,12 +4859,12 @@
       </c>
       <c r="J80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">No lock is needed on the Portal (`PO-25`). Never click Reissue.</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — preconditions restated against `PO-30` (adds the "Ticketed Document" bar, online booking and reissue-capable GDS). Expected result unchanged **only while `PO-25` stands**: `PO-30` condition (5) — locked by the current user — is **Admin-only** (confirmed by the user, 2026-10-01): the Portal has no lock (`PO-25`). Never click Reissue.</t>
         </is>
       </c>
       <c r="K80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L80" t="inlineStr" s="2">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="D82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection (`PO-28`)**, so the button is expected to render.</t>
+          <t xml:space="preserve">**Every `PO-30` condition except the lock holds** — the Portal has no lock and needs none (`PO-25`). AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection**. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). So the button is expected to render.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
@@ -4968,12 +4968,12 @@
       </c>
       <c r="J82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Confirmed intended by the user on 2026-09-24 (FINDING-016, `PO-25`).</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — preconditions restated against `PO-30` (adds the "Ticketed Document" bar, online booking and reissue-capable GDS). Expected result unchanged **only while `PO-25` stands**: `PO-30` condition (5) — locked by the current user — is read as Admin-only; if the reviewer applies it to the Portal, this case's expected result becomes "not shown". Confirmed intended by the user on 2026-09-24 (FINDING-016, `PO-25`).</t>
         </is>
       </c>
       <c r="K82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L82" t="inlineStr" s="2">
@@ -4995,12 +4995,12 @@
       </c>
       <c r="C83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Verify that the Reissue button requires **both** the checkbox on **and** a selected credential matching the credential the PNR was booked on (`PO-28`).</t>
+          <t xml:space="preserve">Verify that the Reissue button requires **both** the checkbox on **and** a selected credential matching the credential the PNR was booked on (`PO-28`, now `PO-30` condition 2).</t>
         </is>
       </c>
       <c r="D83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved), with a selected credential that is **not** the booking's credential — selection is **NDCSabre staging (313)** only, while booking `NDCEG-BR-F260924EAzzYT` is on **Sabre Staging (315)**.</t>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved), with a selected credential that is **not** the booking's credential — selection is **NDCSabre staging (313)** only, while booking `NDCEG-BR-F260924EAzzYT` is on **Sabre Staging (315)**. Every other `PO-30` condition holds: the booking reads Status **Booked** and "Ticketed Document" in the status bar, was made online, is on Sabre (a reissue-capable GDS), and step 5 locks it to you. **Only the credential is unmet.**</t>
         </is>
       </c>
       <c r="F83" t="inlineStr" s="2">
@@ -5025,12 +5025,12 @@
       </c>
       <c r="J83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">**Rev 2, 2026-09-27 — expected result inverted under `PO-28`** (product owner: the button needs the checkbox **and** a selected credential matching the PNR's booking credential). Rev 1 expected "shown" under the now-superseded `PO-22`. Restore AGN9780's selection to include 315 afterwards. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 3, 2026-10-01** — preconditions restated so the credential is the only `PO-30` condition left unmet; the status note now requires the "Ticketed Document" bar too. Expected result unchanged. **Rev 2, 2026-09-27 — expected result inverted under `PO-28`** (product owner: the button needs the checkbox **and** a selected credential matching the PNR's booking credential). Rev 1 expected "shown" under the now-superseded `PO-22`. Restore AGN9780's selection to include 315 afterwards. Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L83" t="inlineStr" s="2">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="D84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A Booked booking made by Admin or the Branch **on behalf of AGN9780**, supplied by the user (`{ONBEHALF_REF}`). BRN265 on, AGN9780 off, both Approved.</t>
+          <t xml:space="preserve">A booking made **online** by Admin or the Branch **on behalf of AGN9780**, supplied by the user (`{ONBEHALF_REF}`), reading Status **Booked** and "Ticketed Document" in the status bar, on a reissue-capable GDS, with its credential in AGN9780's saved selection. BRN265 on, AGN9780 off, both Approved. Step 5 locks it to you, so only AGN9780's checkbox (`PO-30` condition 1) is unmet.</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
@@ -5082,12 +5082,12 @@
       </c>
       <c r="J84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The platform never books; the user supplies `{ONBEHALF_REF}`. Without it, record **Blocked — Awaiting User Booking**. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — preconditions restated against `PO-30`; the status note now requires the "Ticketed Document" bar too. Expected result unchanged. The platform never books; the user supplies `{ONBEHALF_REF}`. Without it, record **Blocked — Awaiting User Booking**. Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L84" t="inlineStr" s="2">
@@ -5104,27 +5104,27 @@
       </c>
       <c r="B85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A booking not in Booked status does not show Reissue</t>
+          <t xml:space="preserve">A booking not both Booked and "Ticketed Document" does not show Reissue</t>
         </is>
       </c>
       <c r="C85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Verify that Reissue is hidden for an Agency booking whose status is not Booked.</t>
+          <t xml:space="preserve">Verify that Reissue is hidden for an Agency booking that does not read **both** Status **Booked** and "Ticketed Document" in the status bar (`PO-30` condition 3).</t>
         </is>
       </c>
       <c r="D85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A booking under AGN9780 in a status other than Booked (e.g. Cancelled), supplied by the user (`{NOTBOOKED_REF}`). AGN9780 on (Approved) **with that booking's credential in the selection (`PO-28`)**, so status is the only condition left unmet.</t>
+          <t xml:space="preserve">A booking under AGN9780 that is **not** Status Booked (the On Hold `{NOTBOOKED_REF}` fixture), supplied by the user. *Optional second booking:* `{BOOKED_UNTICKETED_REF}` — Status **Booked** but the status bar does **not** read "Ticketed Document" — if the user can supply one. AGN9780 on (Approved) **with each booking's credential in the selection**. Each booking was made online on a reissue-capable GDS, and step 5 locks it to you, so condition (3) is the only `PO-30` condition left unmet.</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `{NOTBOOKED_REF}` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `{NOTBOOKED_REF}` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**, and record the Booking Information Status and the status-bar label. | 7. If `{BOOKED_UNTICKETED_REF}` was supplied, repeat steps 3–6 for it.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+          <t xml:space="preserve">The **Reissue** button is not shown for either booking.</t>
         </is>
       </c>
       <c r="H85" t="inlineStr" s="2">
@@ -5139,12 +5139,12 @@
       </c>
       <c r="J85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Without `{NOTBOOKED_REF}`, record **Blocked — Awaiting User Booking**. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — re-aimed at the combined `PO-30` condition (3): Status Booked **and** the "Ticketed Document" bar. Adds the optional Booked-but-not-"Ticketed Document" booking, the half `PO-30` makes new; without it, record that half **Blocked — Awaiting User Booking**. Expected result for `{NOTBOOKED_REF}` unchanged. Without `{NOTBOOKED_REF}`, record **Blocked — Awaiting User Booking**. Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L85" t="inlineStr" s="2">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="D86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off.</t>
+          <t xml:space="preserve">AGN9780 is Approved with Auto Reissue off. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). Step 1 selects its credential and step 7 locks it to you, so only the pending/approved state is under test.</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
@@ -5196,12 +5196,12 @@
       </c>
       <c r="J86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Exploratory: no fixed pass/fail. Opens RSK-013. Never click **Reissue**, **Release PNR** or **Void / Cancel**. Status **Booked** in Booking Information is the condition, not the "Ticketed Document" bar (`PO-24`).</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — preconditions restated against `PO-30`; the status note now requires the "Ticketed Document" bar too. Still exploratory. Exploratory: no fixed pass/fail. Opens RSK-013. Never click **Reissue**, **Release PNR** or **Void / Cancel**. The status condition is Status **Booked** in Booking Information **and** the "Ticketed Document" status bar — both (`PO-30`, which supersedes `PO-24`'s first sentence).</t>
         </is>
       </c>
       <c r="K86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L86" t="inlineStr" s="2">
@@ -5687,17 +5687,17 @@
       </c>
       <c r="C95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Verify that the Portal does not show Reissue for an Agency booking whose status is On Hold.</t>
+          <t xml:space="preserve">Verify that the Portal does not show Reissue for an Agency booking whose status is On Hold — not Status **Booked** with the "Ticketed Document" bar (`PO-30` condition 3).</t>
         </is>
       </c>
       <c r="D95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved) **with that booking's credential in the selection (`PO-28`)**, so status is the only condition left unmet. Booking `NDCEG-BR-F251014N1oohh` (AGN9780, On Hold). The AGN9780 Portal login is available.</t>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved) **with that booking's credential in the selection**. Booking `NDCEG-BR-F251014N1oohh` (AGN9780, On Hold), made online on a reissue-capable GDS. The Portal needs no lock (`PO-25`), so condition (3) is the only `PO-30` condition left unmet. The AGN9780 Portal login is available.</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1. Log in to the Portal (`http://192.168.1.60:9500`) with agency code `AGN9780`. | 2. Open **My Booking** and click **Search**. | 3. Click the **Order Id** of booking `NDCEG-BR-F251014N1oohh`. | 4. Click **View Passenger Details**.</t>
+          <t xml:space="preserve">1. Log in to the Portal (`http://192.168.1.60:9500`) with agency code `AGN9780`. | 2. Open **My Booking** and click **Search**. | 3. Click the **Order Id** of booking `NDCEG-BR-F251014N1oohh`. | 4. Click **View Passenger Details**, and record the status-bar label.</t>
         </is>
       </c>
       <c r="G95" t="inlineStr" s="2">
@@ -5717,15 +5717,186 @@
       </c>
       <c r="J95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Added 2026-09-25 at the user's request ("check the appearance of the button in Admin and Portal"). The Admin side is TC-AGENCY-084. Only Status **Booked** shows Reissue (spec §5, `PO-24`). Never click **Reissue**, **Release PNR** or **Void / Cancel**.</t>
+          <t xml:space="preserve">**Rev 2, 2026-10-01** — re-aimed at the combined `PO-30` condition (3). Expected result unchanged. Added 2026-09-25 at the user's request ("check the appearance of the button in Admin and Portal"). The Admin side is TC-AGENCY-084. Only Status **Booked** together with the "Ticketed Document" status bar shows Reissue (spec §5, `PO-30`). Never click **Reissue**, **Release PNR** or **Void / Cancel**.</t>
         </is>
       </c>
       <c r="K95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Pending</t>
         </is>
       </c>
       <c r="L95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admin hides Reissue for an imported (offline) Agency booking</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Admin Itinerary hides Reissue for an Agency booking that was not made online, when every other condition holds (`PO-30` condition 4).</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A booking under AGN9780 that was **imported** (Import PNR) or made **offline**, supplied by the user (`{OFFLINE_REF}`). It is on Sabre Staging (315) and reads Status **Booked** and "Ticketed Document" in the status bar. AGN9780 has Auto Reissue on (Approved) with 315 in the selection. The booking is not locked by another user; step 5 locks it to you, so only condition (4) is unmet.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `{OFFLINE_REF}` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative, Business-Rule</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Added 2026-10-01 — `PO-30` condition (4) had no case. The platform never books or imports (`PO-19`); without `{OFFLINE_REF}`, record **Blocked — Awaiting User Booking**. Record how the Itinerary shows the booking's source, if it does. Restore AGN9780 to off afterwards. Never click **Reissue**, **Release PNR** or **Void / Cancel**.</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admin shows Reissue only after the booking is locked</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Admin Itinerary hides Reissue until the current user locks the booking (`PO-30` condition 5).</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">AGN9780 has Auto Reissue on (Approved) **with Sabre Staging (315) — the booking's credential — in the selection**. Booking `NDCEG-BR-F260924EAzzYT` (AGN9780, Sabre — a reissue-capable GDS — credential 315) reads Status **Booked** in Booking Information **and** "Ticketed Document" in the status bar, and was made **online** by the user (not offline / imported). It is **not locked by anyone** at the start, so only condition (5) is unmet until step 7.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `NDCEG-BR-F260924EAzzYT` and click **Search**. | 4. Open the booking from the result row. Do **not** click the lock icon. | 5. Click **View Passenger Details**. | 6. Record whether **Reissue** is shown. | 7. Click the lock icon on the **Created By** card. | 8. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">At step 6 the **Reissue** button is not shown. After step 8 it is shown.</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative, Business-Rule</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Added 2026-10-01 — `PO-30` condition (5) had no Admin case. Admin only: the Portal has no lock and needs none (`PO-25`). If the booking is already locked by another user, record **Blocked** and don't take the lock over. Restore AGN9780 to off afterwards. Never click **Reissue**, **Release PNR** or **Void / Cancel**.</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-AGENCY-097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admin hides Reissue for an Agency booking on a supplier that does not support reissue</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Admin Itinerary hides Reissue for an Agency booking whose supplier is not a reissue-capable GDS (`PO-30` condition 6).</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A booking under AGN9780 on a supplier **not** on the reissue list (`NDCsbr`, `Sabre`, `TravelportNdc`, `Galileo`) — e.g. Amadeus or an LCC — supplied by the user (`{NONREISSUE_SUPPLIER_REF}`). It was made online and reads Status **Booked** and "Ticketed Document" in the status bar. AGN9780 has Auto Reissue on (Approved). The booking is not locked by another user; step 5 locks it to you.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open **Booking-Mid Office → Search Booking** (`/booking/search-booking`). | 2. Click the **Flight** tab. | 3. Enter Booking Reference `{NONREISSUE_SUPPLIER_REF}` and click **Search**. | 4. Open the booking from the result row. | 5. Click the lock icon on the **Created By** card. | 6. Click **View Passenger Details**.</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The **Reissue** button is not shown.</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative, Business-Rule</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Added 2026-10-01 — `PO-30` condition (6) had no button case. **Condition (6) cannot be isolated from condition (2) here:** the picker never offers an Amadeus or LCC credential (`PO-21`; TC-BR-085, TC-BR-087), so this booking's credential can't be in AGN9780's selection. The case asserts the outcome both require. The platform never books (`PO-19`); without `{NONREISSUE_SUPPLIER_REF}`, record **Blocked — Awaiting User Booking**. If AGN9780 has no such supplier, ask the user — never change Product Access without asking. Restore AGN9780 to off afterwards. Never click **Reissue**, **Release PNR** or **Void / Cancel**.</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Pending</t>
         </is>

</xml_diff>